<commit_message>
fix(phan-khai-kinh-phi): giữ layout template Excel khi export
Tắt AutoFit cho KetQuaPhanKhaiVonDuocDuyet và cập nhật template (Times New Roman 11, độ rộng cột theo BA).
</commit_message>
<xml_diff>
--- a/QLDA.WebApi/PrintTemplates/KetQuaPhanKhaiVonDuocDuyet.xlsx
+++ b/QLDA.WebApi/PrintTemplates/KetQuaPhanKhaiVonDuocDuyet.xlsx
@@ -1,157 +1,84 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SER\QLDA.WebApi\PrintTemplates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82067616-CAF9-4CB6-8CED-BA9EAFB0F815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="KetQuaPhanKhaiVon" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KetQuaPhanKhaiVon" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
-  <si>
-    <t>KẾT QUẢ PHÂN KHAI VỐN ĐƯỢC DUYỆT</t>
-  </si>
-  <si>
-    <t>STT</t>
-  </si>
-  <si>
-    <t>Số tờ trình</t>
-  </si>
-  <si>
-    <t>Trích yếu</t>
-  </si>
-  <si>
-    <t>Nguồn</t>
-  </si>
-  <si>
-    <t>KP đề xuất (tr)</t>
-  </si>
-  <si>
-    <t>KP phân khai (tr)</t>
-  </si>
-  <si>
-    <t>Trạng thái</t>
-  </si>
-  <si>
-    <t>Thao tác</t>
-  </si>
-  <si>
-    <t>$Stt</t>
-  </si>
-  <si>
-    <t>$SoToTrinh</t>
-  </si>
-  <si>
-    <t>$TrichYeu</t>
-  </si>
-  <si>
-    <t>$TenNguonVon</t>
-  </si>
-  <si>
-    <t>$KinhPhiDeXuat</t>
-  </si>
-  <si>
-    <t>$KinhPhiPhanKhai</t>
-  </si>
-  <si>
-    <t>$TenTrangThai</t>
-  </si>
-  <si>
-    <t>$ThaoTac</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">
-TRUNG TÂM CHUYỂN ĐỔI SỐ </t>
-    </r>
-  </si>
-  <si>
-    <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
-Độc lập - Tự do - Hạnh phúc
----------------</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
+  <fonts count="10">
+    <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
+      <b val="1"/>
       <sz val="11"/>
-      <color theme="1"/>
+    </font>
+    <font>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <b/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
+    </font>
+    <font>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
+      <b val="1"/>
       <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
+      <b val="1"/>
       <color theme="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -161,8 +88,13 @@
         <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -194,46 +126,168 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="30">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -521,124 +575,145 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" style="10" customWidth="1"/>
-    <col min="2" max="2" width="15" style="10" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" style="10" customWidth="1"/>
-    <col min="4" max="4" width="59.6640625" style="10" customWidth="1"/>
-    <col min="5" max="5" width="22.5546875" style="10" customWidth="1"/>
-    <col min="6" max="6" width="26.6640625" style="10" customWidth="1"/>
-    <col min="7" max="7" width="38.5546875" style="10" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" style="10" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="10"/>
+    <col width="6.89" customWidth="1" style="3" min="1" max="1"/>
+    <col width="14.22" customWidth="1" style="3" min="2" max="2"/>
+    <col width="80.67" customWidth="1" style="3" min="3" max="3"/>
+    <col width="17.89" customWidth="1" style="3" min="4" max="4"/>
+    <col width="21.78" customWidth="1" style="3" min="5" max="5"/>
+    <col width="25.89" customWidth="1" style="3" min="6" max="6"/>
+    <col width="20.44" customWidth="1" style="3" min="7" max="7"/>
+    <col width="8.88671875" customWidth="1" style="3" min="8" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
+TRUNG TÂM CHUYỂN ĐỔI SỐ </t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
+Độc lập - Tự do - Hạnh phúc
+---------------</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="n"/>
+      <c r="I1" s="4" t="n"/>
+      <c r="J1" s="4" t="n"/>
     </row>
-    <row r="2" spans="1:11" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
+    <row r="2" ht="13.2" customHeight="1">
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="4" t="n"/>
+      <c r="J2" s="4" t="n"/>
     </row>
-    <row r="3" spans="1:11" ht="22.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
+    <row r="3" ht="22.8" customHeight="1">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>KẾT QUẢ PHÂN KHAI VỐN ĐƯỢC DUYỆT</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>8</v>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Số tờ trình</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>Trích yếu</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>Nguồn</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>KP đề xuất (tr)</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>KP phân khai (tr)</t>
+        </is>
+      </c>
+      <c r="G4" s="26" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>16</v>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>$Stt</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>$SoToTrinh</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>$TrichYeu</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>$TenNguonVon</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="inlineStr">
+        <is>
+          <t>$KinhPhiDeXuat</t>
+        </is>
+      </c>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>$KinhPhiPhanKhai</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>$TenTrangThai</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="A3:G3"/>
     <mergeCell ref="A1:D2"/>
-    <mergeCell ref="E1:H2"/>
-    <mergeCell ref="A3:H3"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>